<commit_message>
Inicio de limpieza, nada relevante
</commit_message>
<xml_diff>
--- a/Template.xlsx
+++ b/Template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EPV\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\D'Aaron\Curso de Python\Hymn_List_Manager\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,124 +24,232 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="73">
   <si>
     <t>R</t>
   </si>
   <si>
-    <t>TE LOAMOS O DIOS</t>
-  </si>
-  <si>
-    <t>SANTO SANTO SANTO</t>
-  </si>
-  <si>
-    <t>COMO PODRE ESTAR TRISTE</t>
-  </si>
-  <si>
-    <t>HALLE UN BUEN AMIGO</t>
-  </si>
-  <si>
-    <t>CUAN GRANDE ES EL</t>
-  </si>
-  <si>
-    <t>PECADOR VEN A CRISTO JESUS</t>
-  </si>
-  <si>
-    <t>LUCHANDO ESTAIS</t>
-  </si>
-  <si>
-    <t>LOORES DAD A CRSITO EL REY</t>
-  </si>
-  <si>
-    <t>FIRMES Y ADELANTE</t>
-  </si>
-  <si>
-    <t>DIRE A CRISTO</t>
-  </si>
-  <si>
-    <t>ME GUIA EL</t>
-  </si>
-  <si>
-    <t>LA NUEVA PROCLAMAD</t>
-  </si>
-  <si>
-    <t>AL MUNDO PAZ NACIO JESUS</t>
-  </si>
-  <si>
-    <t>CASTILLO FUERTE</t>
-  </si>
-  <si>
-    <t>SANTA BIBLIA PARA MI</t>
-  </si>
-  <si>
-    <t>SEMBRARE LA SIMIENTE PRECIOSO</t>
-  </si>
-  <si>
-    <t>SE OYE UN SON EN ALTA ESFERA</t>
-  </si>
-  <si>
-    <t>GOZO LA SANTA PALABRA AL LEER</t>
-  </si>
-  <si>
-    <t>AMA A TUS PROJIMOS</t>
-  </si>
-  <si>
-    <t>ALCANCE SALVACION</t>
-  </si>
-  <si>
-    <t>GRACIA ADMIRABLE</t>
-  </si>
-  <si>
-    <t>PON TUS OJOS EN CRISTO</t>
-  </si>
-  <si>
-    <t>SE TU MI VISION</t>
-  </si>
-  <si>
-    <t>LAS PISADAS DEL MAESTRO</t>
-  </si>
-  <si>
-    <t>ME AGRADA CANTAR</t>
-  </si>
-  <si>
-    <t>EL REY YA VIENE</t>
-  </si>
-  <si>
-    <t>TAL COMO ES HOY</t>
-  </si>
-  <si>
-    <t>CRISTO SOSTENDRA</t>
-  </si>
-  <si>
-    <t>NADIE PUDO AMARME COMO CRISTO</t>
-  </si>
-  <si>
-    <t>TODO LO PAGO</t>
-  </si>
-  <si>
-    <t>VISTE TU</t>
-  </si>
-  <si>
-    <t>DIOS OS GUARDE</t>
-  </si>
-  <si>
-    <t>TUYO SOY SEÑOR</t>
-  </si>
-  <si>
-    <t>QUE TODO EL MUNDO CANTE</t>
-  </si>
-  <si>
-    <t>HAY UN PRECIOSO MANANTIAL</t>
-  </si>
-  <si>
-    <t>(fecha: debe contener un numero)</t>
+    <t>todo lo pago</t>
+  </si>
+  <si>
+    <t>la tumba le encerro</t>
+  </si>
+  <si>
+    <t>gracia admirable</t>
+  </si>
+  <si>
+    <t>oh que tuviera lenguas mil</t>
+  </si>
+  <si>
+    <t>cual pendon hermoso</t>
+  </si>
+  <si>
+    <t>te necesito ya</t>
+  </si>
+  <si>
+    <t>cuando alla se pase lista</t>
+  </si>
+  <si>
+    <t>grato es contar la historia</t>
+  </si>
+  <si>
+    <t>santo santo santo</t>
+  </si>
+  <si>
+    <t>grande es contar la historia</t>
+  </si>
+  <si>
+    <t>viste tu</t>
+  </si>
+  <si>
+    <t>victoria en crsito</t>
+  </si>
+  <si>
+    <t>te loamos oh Dios</t>
+  </si>
+  <si>
+    <t>aleluya gloria a cristo</t>
+  </si>
+  <si>
+    <t>en jesucristo el reyu depaz</t>
+  </si>
+  <si>
+    <t>prefiero a crsito</t>
+  </si>
+  <si>
+    <t>cerca de ti señor</t>
+  </si>
+  <si>
+    <t>el profundo amor de cristo</t>
+  </si>
+  <si>
+    <t>bendecido el gran manantial</t>
+  </si>
+  <si>
+    <t>Canten del amor de cristo</t>
+  </si>
+  <si>
+    <t>alcristovivosirvo</t>
+  </si>
+  <si>
+    <t>el muno es de miDios</t>
+  </si>
+  <si>
+    <t>Todolopago</t>
+  </si>
+  <si>
+    <t>sugraciaesmayor</t>
+  </si>
+  <si>
+    <t>todas laspromesadelseñor</t>
+  </si>
+  <si>
+    <t>maravillosoeselgranamor</t>
+  </si>
+  <si>
+    <t>gratoescontarlahistoria</t>
+  </si>
+  <si>
+    <t>cristodivinohiojubigenito</t>
+  </si>
+  <si>
+    <t>pontusojosescristo</t>
+  </si>
+  <si>
+    <t>lejosdemipadredios</t>
+  </si>
+  <si>
+    <t>talcomoeshoy</t>
+  </si>
+  <si>
+    <t>looresdadacrsitoelrey</t>
+  </si>
+  <si>
+    <t>tengoanteeltrono</t>
+  </si>
+  <si>
+    <t>grandestufidewlidad</t>
+  </si>
+  <si>
+    <t>prefieroacrsito</t>
+  </si>
+  <si>
+    <t>graciaadmirable</t>
+  </si>
+  <si>
+    <t>firmesyadelante</t>
+  </si>
+  <si>
+    <t>almabendicealseñor</t>
+  </si>
+  <si>
+    <t>castillofuerteesnuestrodios</t>
+  </si>
+  <si>
+    <t>aleluyagloriaacristo</t>
+  </si>
+  <si>
+    <t>señorjesuslaluzdelsolsefue</t>
+  </si>
+  <si>
+    <t>elprofundoamordecristo</t>
+  </si>
+  <si>
+    <t>cristodivinohijounigenito</t>
+  </si>
+  <si>
+    <t>hayunnombrenuevoenlagloria</t>
+  </si>
+  <si>
+    <t>dois os guarde</t>
+  </si>
+  <si>
+    <t>fuente de la vida eterna</t>
+  </si>
+  <si>
+    <t>anhelotrabajar por el señor</t>
+  </si>
+  <si>
+    <t>maravillososeselgranamor</t>
+  </si>
+  <si>
+    <t>enlacruz</t>
+  </si>
+  <si>
+    <t>no cambiara</t>
+  </si>
+  <si>
+    <t>en el monte calvario</t>
+  </si>
+  <si>
+    <t>alcance salvacion</t>
+  </si>
+  <si>
+    <t>todas las promesas del señor</t>
+  </si>
+  <si>
+    <t>halle un buen amigo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">maravilloso es </t>
+  </si>
+  <si>
+    <t>lojos de mi padre dios</t>
+  </si>
+  <si>
+    <t>estad por cristo firmes</t>
+  </si>
+  <si>
+    <t>castillo fiuerte es nuestro Dios</t>
+  </si>
+  <si>
+    <t>hay un precioso manantial</t>
+  </si>
+  <si>
+    <t>lluvias de rgacia</t>
+  </si>
+  <si>
+    <t>te loamos oh dios</t>
+  </si>
+  <si>
+    <t>por que el vice</t>
+  </si>
+  <si>
+    <t>en jesucrsito el rey de paz</t>
+  </si>
+  <si>
+    <t>al crsito vivo9 sirvo</t>
+  </si>
+  <si>
+    <t>viene otravez</t>
+  </si>
+  <si>
+    <t>amigo halle</t>
+  </si>
+  <si>
+    <t>cerca de ti</t>
+  </si>
+  <si>
+    <t>oh que tuviera lenbguas mil</t>
+  </si>
+  <si>
+    <t>que lindo es cantar</t>
+  </si>
+  <si>
+    <t>en la cruz</t>
+  </si>
+  <si>
+    <t>su gracia es mayor</t>
+  </si>
+  <si>
+    <t>mi vida di por ti.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -162,8 +270,34 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -188,8 +322,38 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFD9"/>
+        <bgColor rgb="FFE2EFD9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -212,11 +376,54 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -233,6 +440,27 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -513,7 +741,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:I24"/>
+  <dimension ref="B2:I40"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -526,20 +754,22 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="4" t="s">
-        <v>36</v>
+      <c r="B2" s="4">
+        <v>3</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>0</v>
       </c>
       <c r="E2" s="5">
-        <v>12</v>
+        <f>B2+4</f>
+        <v>7</v>
       </c>
       <c r="F2" s="6" t="s">
         <v>0</v>
       </c>
       <c r="H2" s="5">
-        <v>18</v>
+        <f>E2</f>
+        <v>7</v>
       </c>
       <c r="I2" s="6" t="s">
         <v>0</v>
@@ -547,289 +777,471 @@
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="C3" s="7"/>
       <c r="E3" s="2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F3" s="7"/>
       <c r="H3" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="I3" s="7"/>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="C4" s="7"/>
       <c r="E4" s="2" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F4" s="7"/>
       <c r="H4" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I4" s="7"/>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="C5" s="7"/>
       <c r="E5" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F5" s="7"/>
       <c r="H5" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I5" s="7"/>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="C6" s="7"/>
       <c r="E6" s="2" t="s">
-        <v>35</v>
+        <v>11</v>
       </c>
       <c r="F6" s="7"/>
       <c r="H6" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I6" s="7"/>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
-        <v>5</v>
+        <v>24</v>
       </c>
       <c r="C7" s="7"/>
       <c r="E7" s="2" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="F7" s="7"/>
       <c r="H7" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I7" s="7"/>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="C8" s="7"/>
       <c r="E8" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F8" s="7"/>
       <c r="H8" s="2" t="s">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="I8" s="7"/>
     </row>
     <row r="10" spans="2:9" s="1" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="5">
-        <v>20</v>
+        <f>B2+7</f>
+        <v>10</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>0</v>
       </c>
       <c r="E10" s="5">
-        <v>25</v>
+        <f>B10+4</f>
+        <v>14</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>0</v>
       </c>
       <c r="H10" s="5">
-        <v>30</v>
-      </c>
-      <c r="I10" s="6"/>
+        <f>E10</f>
+        <v>14</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B11" s="2" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="C11" s="7"/>
       <c r="E11" s="2" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="F11" s="7"/>
       <c r="H11" s="2" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="I11" s="7"/>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B12" s="2" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="C12" s="7"/>
       <c r="E12" s="2" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="F12" s="7"/>
       <c r="H12" s="2" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="I12" s="7"/>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B13" s="2" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="C13" s="7"/>
       <c r="E13" s="2" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="F13" s="7"/>
       <c r="H13" s="2" t="s">
-        <v>14</v>
+        <v>40</v>
       </c>
       <c r="I13" s="7"/>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="C14" s="7"/>
       <c r="E14" s="2" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="F14" s="7"/>
       <c r="H14" s="2" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="I14" s="7"/>
     </row>
     <row r="15" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B15" s="2" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="C15" s="7"/>
       <c r="E15" s="2" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="F15" s="7"/>
       <c r="H15" s="2" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="I15" s="7"/>
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B16" s="2" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="C16" s="7"/>
       <c r="E16" s="2" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="F16" s="7"/>
       <c r="H16" s="2" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="I16" s="7"/>
     </row>
     <row r="18" spans="2:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="5">
-        <v>20</v>
-      </c>
-      <c r="C18" s="6"/>
+        <f>B10+7</f>
+        <v>17</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>0</v>
+      </c>
       <c r="D18" s="1"/>
       <c r="E18" s="5">
-        <v>25</v>
-      </c>
-      <c r="F18" s="6"/>
+        <f>B18+4</f>
+        <v>21</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>0</v>
+      </c>
       <c r="G18" s="1"/>
       <c r="H18" s="5">
-        <v>30</v>
-      </c>
-      <c r="I18" s="6"/>
+        <f>E18</f>
+        <v>21</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B19" s="2" t="s">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="C19" s="7"/>
-      <c r="E19" s="2" t="s">
-        <v>26</v>
+      <c r="E19" s="8" t="s">
+        <v>48</v>
       </c>
       <c r="F19" s="7"/>
-      <c r="H19" s="2" t="s">
-        <v>33</v>
+      <c r="H19" s="9" t="s">
+        <v>54</v>
       </c>
       <c r="I19" s="7"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B20" s="2" t="s">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="C20" s="7"/>
-      <c r="E20" s="2" t="s">
-        <v>27</v>
+      <c r="E20" s="9" t="s">
+        <v>49</v>
       </c>
       <c r="F20" s="7"/>
-      <c r="H20" s="2" t="s">
-        <v>34</v>
+      <c r="H20" s="12" t="s">
+        <v>6</v>
       </c>
       <c r="I20" s="7"/>
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B21" s="2" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="C21" s="7"/>
-      <c r="E21" s="2" t="s">
-        <v>28</v>
+      <c r="E21" s="10" t="s">
+        <v>50</v>
       </c>
       <c r="F21" s="7"/>
-      <c r="H21" s="2" t="s">
-        <v>14</v>
+      <c r="H21" s="13" t="s">
+        <v>55</v>
       </c>
       <c r="I21" s="7"/>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B22" s="2" t="s">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="C22" s="7"/>
-      <c r="E22" s="2" t="s">
-        <v>29</v>
+      <c r="E22" s="9" t="s">
+        <v>51</v>
       </c>
       <c r="F22" s="7"/>
-      <c r="H22" s="2" t="s">
-        <v>30</v>
+      <c r="H22" s="14" t="s">
+        <v>56</v>
       </c>
       <c r="I22" s="7"/>
     </row>
     <row r="23" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B23" s="2" t="s">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="C23" s="7"/>
-      <c r="E23" s="2" t="s">
-        <v>25</v>
+      <c r="E23" s="8" t="s">
+        <v>52</v>
       </c>
       <c r="F23" s="7"/>
-      <c r="H23" s="2" t="s">
-        <v>31</v>
+      <c r="H23" s="15" t="s">
+        <v>11</v>
       </c>
       <c r="I23" s="7"/>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B24" s="2" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C24" s="7"/>
-      <c r="E24" s="2" t="s">
+      <c r="E24" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="F24" s="7"/>
+      <c r="H24" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="I24" s="7"/>
+    </row>
+    <row r="26" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B26" s="5">
+        <f>B18+7</f>
         <v>24</v>
       </c>
-      <c r="F24" s="7"/>
-      <c r="H24" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="I24" s="7"/>
+      <c r="C26" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="D26" s="1"/>
+      <c r="E26" s="5">
+        <f>B26+4</f>
+        <v>28</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="G26" s="1"/>
+      <c r="H26" s="5">
+        <f>E26</f>
+        <v>28</v>
+      </c>
+      <c r="I26" s="6" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B27" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C27" s="7"/>
+      <c r="E27" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="F27" s="7"/>
+      <c r="H27" s="23" t="s">
+        <v>5</v>
+      </c>
+      <c r="I27" s="7"/>
+    </row>
+    <row r="28" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B28" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="C28" s="7"/>
+      <c r="E28" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="F28" s="7"/>
+      <c r="H28" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="I28" s="7"/>
+    </row>
+    <row r="29" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B29" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="C29" s="7"/>
+      <c r="E29" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="F29" s="7"/>
+      <c r="H29" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="I29" s="7"/>
+    </row>
+    <row r="30" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B30" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="C30" s="7"/>
+      <c r="E30" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="F30" s="7"/>
+      <c r="H30" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="I30" s="7"/>
+    </row>
+    <row r="31" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B31" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="C31" s="7"/>
+      <c r="E31" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="F31" s="7"/>
+      <c r="H31" s="24" t="s">
+        <v>67</v>
+      </c>
+      <c r="I31" s="7"/>
+    </row>
+    <row r="32" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B32" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="C32" s="7"/>
+      <c r="E32" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="F32" s="7"/>
+      <c r="H32" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="I32" s="7"/>
+    </row>
+    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B34" s="5">
+        <f>B26+7</f>
+        <v>31</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="E34" s="5"/>
+      <c r="F34" s="6"/>
+    </row>
+    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B35" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C35" s="7"/>
+      <c r="E35" s="2"/>
+      <c r="F35" s="7"/>
+    </row>
+    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B36" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="C36" s="7"/>
+      <c r="E36" s="2"/>
+      <c r="F36" s="7"/>
+    </row>
+    <row r="37" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B37" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="C37" s="7"/>
+      <c r="E37" s="2"/>
+      <c r="F37" s="7"/>
+    </row>
+    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B38" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="C38" s="7"/>
+      <c r="E38" s="2"/>
+      <c r="F38" s="7"/>
+    </row>
+    <row r="39" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B39" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="C39" s="7"/>
+      <c r="E39" s="2"/>
+      <c r="F39" s="7"/>
+    </row>
+    <row r="40" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B40" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="C40" s="7"/>
+      <c r="E40" s="2"/>
+      <c r="F40" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>